<commit_message>
feat: build dynamic project intelligence MVP
</commit_message>
<xml_diff>
--- a/data/raw/betavanx_mvp_v1.xlsx
+++ b/data/raw/betavanx_mvp_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SINA\Desktop\شروع داستان\BeTavaneX\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF85A9F4-5A2D-45E1-85E8-A8B18E0D0269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A25EA3B8-EE41-463B-9B4B-D72C618834EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10718" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-83" yWindow="0" windowWidth="13126" windowHeight="12863" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="29">
   <si>
     <t>id</t>
   </si>
@@ -116,6 +116,9 @@
   </si>
   <si>
     <t>amount</t>
+  </si>
+  <si>
+    <t>baseline_qty</t>
   </si>
 </sst>
 </file>
@@ -468,16 +471,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.73046875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.19921875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.9296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -490,8 +494,11 @@
       <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E1" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -503,6 +510,9 @@
       </c>
       <c r="D2" s="6">
         <v>5000000</v>
+      </c>
+      <c r="E2" s="1">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>